<commit_message>
test(qa): REL-15 회귀 시트 40행 완결 — WY-qa2 10행 합침(R15-50~59 모두 PASS), R15-12는 3b64945 수정을 로컬 mock에서 1280·390 재검증해 PASS(운영 재확인은 REL-18 배포 뒤)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/REL-15_회귀시트_v1.0.xlsx
+++ b/docs/qa/REL-15_회귀시트_v1.0.xlsx
@@ -932,22 +932,22 @@
       <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">빈 제출·형식 오류 모두 칸 오류(aria-invalid, "입력해 주세요"/"이메일 형식이 맞지 않아요")는 뜨나 포커스가 [인증번호 받기] 버튼에 남음. 발송 요청 0</t>
+          <t xml:space="preserve">운영(8c8f1a8)에서는 빈 제출·형식 오류 모두 칸 오류는 뜨나 포커스가 [인증번호 받기]에 남음(FAIL, forgot-*-1280.png). 수정 3b64945를 로컬 mock으로 재검증: 찾기 빈 제출·not-an-email 모두 이메일 칸 포커스+aria-invalid, 재설정 저장 단계 새 비밀번호 규칙 위반→새 비밀번호 칸, 둘 다 틀림→새 비밀번호 칸, 확인 불일치→확인 칸, 1280·390 모두</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIL</t>
+          <t xml:space="preserve">PASS(로컬 재검증)</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">forgot-error-1280.png, forgot-focus-1280.png</t>
+          <t xml:space="preserve">forgot-error-1280.png, forgot-focus-1280.png(운영 FAIL) · r1512-forgot-1280.png, r1512-forgot-390.png, r1512-reset-pw-1280.png, r1512-reset-pw-390.png, r1512-reset-confirm-1280.png, r1512-reset-confirm-390.png(로컬)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">메일 발송은 pm 승인 후 별도 / [결함] 낮음~중간, 화면정의서 2.5 REL-09 규칙(첫 오류 칸 포커스) 미적용. pm 보고함</t>
+          <t xml:space="preserve">메일 발송은 pm 승인 후 별도 / [결함] 수정됨(3b64945, feature/REL). 운영 재확인은 REL-18 배포 뒤. 재설정 메일 발송 단계는 누르지 않음</t>
         </is>
       </c>
     </row>
@@ -1950,9 +1950,21 @@
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M/W/D 키와 보기 링크로 월·주·일 전환, 이전·다음·오늘 이동 정상, 390 가로 넘침 없음, 콘솔 오류 0. 참고: 월 보기에서 D를 누르면 그 달 1일의 일 보기로 감(URL이 /month/YYYY-MM이라 일자가 없음, 오늘이 그 달에 있어도 1일)</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-50-week-1280.png · R15-50-month-1280.png · R15-50-day-1280.png · R15-50-week-390.png · R15-50-month-390.png · R15-50-day-390.png</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1992,9 +2004,21 @@
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">매주 반복 일정 생성 토스트·수정 시 범위 창(이 일정만/모든 일정) 확인·삭제 후 토스트 [되돌리기] 44px로 복원·끌어 옮기기(23:00→21:15, 옮김 확인 창+토스트) 정상. 겹침 12개는 12열로 나뉘고(1280 폭 18px·390 폭 20px, 중심 간격 24px 안팎) 가로 넘침 없음, 블록 안 글자는 읽기 어렵고 접근 이름(aria-label)으로 구분</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-51-create-repeat.png · R15-51-edit-scope.png · R15-51-overlap12-1280.png · R15-51-overlap12-390.png</t>
+        </is>
+      </c>
       <c r="L32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
@@ -2038,9 +2062,21 @@
           <t xml:space="preserve">R15-19~R15-21</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">옵션 꺼짐·켜짐 모두 행에 "계획 09:30 – 10:30" 표시. 옵션 켠 상태 수정 창 시간 칸 09:30~10:30(1280·390), 일정 상세 [기록 보기]에서 연 창도 09:30~10:30. 옵션 꺼짐 상태에서는 시간 칸 자체가 숨겨짐(기록 날짜만)</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-52-pending-edit-1280.png · R15-52-pending-edit-timeon-1280.png · R15-52-pending-edit-390.png</t>
+        </is>
+      </c>
       <c r="L33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2084,9 +2120,21 @@
           <t xml:space="preserve">R15-24</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">오늘 끝나지 않은 일정 상세에서 [이 일정으로 타이머 시작] 정상. 1분 미만 정지는 안내 토스트와 함께 계획이 확인 대기로 돌아감, 1분 넘겨 정지하면 "기록을 남겼어요". 오프라인 전환 시 "연결 끊김" 표시·정지 버튼 비활성, 복귀 후 해제. 끝난 일정(10-11 09:30)에는 타이머 시작 버튼 없음</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-53-timer-running-1280.png · R15-53-timer-offline-1280.png</t>
+        </is>
+      </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">계정 상태를 바꿈 — qa2만</t>
@@ -2130,9 +2178,21 @@
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3단계(1/3 확인 대기 처리 → 2/3 다음 근무일 계획 이월 → 3/3 이슈·마감하고 확정, 시트의 "2단계" 문구는 낡음). 확인 대기 [했어요] 후 토스트·이월 목록·다음 근무일 10/13(화), 확정 직전 작성자 정보 창(앞서 [나중에]한 뒤 한 번 더 묻는 규칙) → [나중에] → "오늘 일지를 확정했어요", 일지 확정 표시. [확정 해제]로 초안 복원(해제 뒤 표시가 "실적 고정"으로 바뀜, 내용은 그대로)</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-54-step1-1280.png · R15-54-step3-1280.png · R15-54-confirm-1280.png · R15-54-confirmed-log-1280.png</t>
+        </is>
+      </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">계정 상태를 바꿈 — qa2만, 확정 해제로 원복</t>
@@ -2176,9 +2236,21 @@
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일지 목록(월 달력)·일간·주간·월간 상세 모두 열림, 열기 약 0.9~1.0초(월간 포함), 390 가로 넘침 없음, 콘솔 오류 0. 처음 여는 일지에서 작성자 정보 창이 한 번 뜸(규칙대로)</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-55-daily_2026-10-07-1280.png · R15-55-weekly_2026-10-05-1280.png · R15-55-monthly_2026-10-1280.png · 같은 이름 -390.png</t>
+        </is>
+      </c>
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
@@ -2218,9 +2290,21 @@
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">일간 일지 10-06: 업무일지_2026-10-06.pdf/.docx/.xlsx 생성(파일 머리 25 50 44 46 / 50 4B 03 04 / 50 4B 03 04, MIME 정상), 토스트 "파일을 내려받았어요". 주간 10-05: 업무일지_2026-10-05.pdf/.xlsx. 파일은 앱에서 만든 blob을 가로채 확인(내려받은 파일을 프로그램으로 열어 보지는 않음)</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (blob 가로채기 결과)</t>
+        </is>
+      </c>
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2264,9 +2348,21 @@
           <t xml:space="preserve">R15-18</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기록이 7일 미만인 B 계정은 "1주일 기록이 쌓이면" 안내만 보여 과거 날짜 시험 기록 3건을 만든 뒤 확인(끝나고 삭제). 이번 주·이번 달·직접 선택 10/1–10/31(종료일 미래)·최근 3개월 7/12–10/11 모두 요약·주별/달별 막대 표시, 소요시간 비중 표시, 390 가로 넘침 없음, 콘솔 오류 0. 시트의 "최근 3개월"은 빠른 선택 칩은 [직접 선택] 안에 있음(최상단은 이번 주·이번 달·직접 선택)</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-57-stats-1280.png · R15-57-stats-390.png</t>
+        </is>
+      </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">기록이 쌓인 계정에서</t>
@@ -2310,9 +2406,21 @@
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보관 시각 내림차순 정렬. [복원] 후 목록에서 빠지고 토스트 [보기] 44×44(업무 상세로 이동)·[되돌리기] 80×44, 되돌리면 목록에 다시 나타남(1280·390 모두)</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R15-58-archive-390.png</t>
+        </is>
+      </c>
       <c r="L39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2352,9 +2460,21 @@
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 터치 입력(CDP Input.dispatchTouchEvent): 블록 위에서 세로로 밀면 격자 스크롤 227→529px만 바뀌고 일정·창 변화 없음. 650ms 길게 누른 뒤 아래로 끌면 10:00→12:00으로 옮겨지고 "일정을 옮겼어요" 토스트, 스크롤 그대로</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">— (스크립트 결과)</t>
+        </is>
+      </c>
       <c r="L40" s="2" t="inlineStr"/>
     </row>
     <row r="41">

</xml_diff>